<commit_message>
Shows März + Eintritte und Kiosk Brutalist 2.3.25
</commit_message>
<xml_diff>
--- a/Input/Spezialpreisekiosk.xlsx
+++ b/Input/Spezialpreisekiosk.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\R Packages\Kinoklub\Input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kinoklub\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11EEBD71-3D11-487B-933A-9EF0081FB841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13C79F4D-398E-43BA-A7F7-171F37876A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4740" yWindow="4890" windowWidth="24225" windowHeight="12975" xr2:uid="{5CFCAA73-5DB4-4EB4-81C9-1C9C0D98D4AD}"/>
+    <workbookView xWindow="1820" yWindow="1820" windowWidth="15100" windowHeight="12710" xr2:uid="{5CFCAA73-5DB4-4EB4-81C9-1C9C0D98D4AD}"/>
   </bookViews>
   <sheets>
     <sheet name="Spezpreise" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="15">
   <si>
     <t>Datum</t>
   </si>
@@ -75,6 +75,12 @@
   </si>
   <si>
     <t>1020.643</t>
+  </si>
+  <si>
+    <t>1021.270</t>
+  </si>
+  <si>
+    <t>Gipfeli</t>
   </si>
 </sst>
 </file>
@@ -138,7 +144,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -161,8 +167,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9A44B4B4-A546-4A04-B7DF-39B4610A3FD4}" name="Table1" displayName="Table1" ref="A1:D7" totalsRowShown="0">
-  <autoFilter ref="A1:D7" xr:uid="{9A44B4B4-A546-4A04-B7DF-39B4610A3FD4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9A44B4B4-A546-4A04-B7DF-39B4610A3FD4}" name="Table1" displayName="Table1" ref="A1:D9" totalsRowShown="0">
+  <autoFilter ref="A1:D9" xr:uid="{9A44B4B4-A546-4A04-B7DF-39B4610A3FD4}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D2">
     <sortCondition ref="A1:A2"/>
   </sortState>
@@ -177,9 +183,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 – 2022">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -217,7 +223,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 – 2022">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -323,7 +329,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 – 2022">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -473,16 +479,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD21FE1F-65EF-43DF-AD1F-FCA81656A71F}">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" customWidth="1"/>
+    <col min="1" max="1" width="14.1796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.1796875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="14.7265625" customWidth="1"/>
+    <col min="4" max="4" width="17.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -496,7 +502,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>45676</v>
       </c>
@@ -510,7 +516,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>45683</v>
       </c>
@@ -524,7 +530,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>45690</v>
       </c>
@@ -538,7 +544,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>45690</v>
       </c>
@@ -552,7 +558,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>45701</v>
       </c>
@@ -566,7 +572,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>45683</v>
       </c>
@@ -578,6 +584,34 @@
       </c>
       <c r="D7" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="1">
+        <v>45718</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="1">
+        <v>45718</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Filmvorführung Heldin 2. Vorstellung 10.4.25 Kiosk und Eintritte Wunderschöner 11.4.25 Eintritte und Kiosk Spez Preis Sauvage
</commit_message>
<xml_diff>
--- a/Input/Spezialpreisekiosk.xlsx
+++ b/Input/Spezialpreisekiosk.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kinoklub\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61DA1BDA-2C95-4623-8D62-54090613BE69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D96486A-AE1F-4A5E-8ADB-7C7EAFD853E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11340" yWindow="2440" windowWidth="15100" windowHeight="12710" xr2:uid="{5CFCAA73-5DB4-4EB4-81C9-1C9C0D98D4AD}"/>
+    <workbookView xWindow="340" yWindow="340" windowWidth="22710" windowHeight="14340" xr2:uid="{5CFCAA73-5DB4-4EB4-81C9-1C9C0D98D4AD}"/>
   </bookViews>
   <sheets>
     <sheet name="Spezpreise" sheetId="1" r:id="rId1"/>
@@ -98,7 +98,7 @@
     <t>1020.846</t>
   </si>
   <si>
-    <t>1012.952</t>
+    <t>1018.523</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Eintritte Kiosk und Spezpreise Friedas Fall 13.4.25
</commit_message>
<xml_diff>
--- a/Input/Spezialpreisekiosk.xlsx
+++ b/Input/Spezialpreisekiosk.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kinoklub\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D96486A-AE1F-4A5E-8ADB-7C7EAFD853E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFF6B17F-093B-46C0-A355-7255F63AA72C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="340" yWindow="340" windowWidth="22710" windowHeight="14340" xr2:uid="{5CFCAA73-5DB4-4EB4-81C9-1C9C0D98D4AD}"/>
+    <workbookView xWindow="340" yWindow="340" windowWidth="26870" windowHeight="16160" xr2:uid="{5CFCAA73-5DB4-4EB4-81C9-1C9C0D98D4AD}"/>
   </bookViews>
   <sheets>
     <sheet name="Spezpreise" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="22">
   <si>
     <t>Datum</t>
   </si>
@@ -99,6 +99,9 @@
   </si>
   <si>
     <t>1018.523</t>
+  </si>
+  <si>
+    <t>1019.535</t>
   </si>
 </sst>
 </file>
@@ -193,8 +196,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9A44B4B4-A546-4A04-B7DF-39B4610A3FD4}" name="Table1" displayName="Table1" ref="A1:D13" totalsRowShown="0">
-  <autoFilter ref="A1:D13" xr:uid="{9A44B4B4-A546-4A04-B7DF-39B4610A3FD4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9A44B4B4-A546-4A04-B7DF-39B4610A3FD4}" name="Table1" displayName="Table1" ref="A1:D15" totalsRowShown="0">
+  <autoFilter ref="A1:D15" xr:uid="{9A44B4B4-A546-4A04-B7DF-39B4610A3FD4}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D2">
     <sortCondition ref="A1:A2"/>
   </sortState>
@@ -505,7 +508,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD21FE1F-65EF-43DF-AD1F-FCA81656A71F}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.1796875" style="1" customWidth="1"/>
@@ -696,6 +699,34 @@
         <v>16</v>
       </c>
     </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="1">
+        <v>45760</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="1">
+        <v>45760</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>